<commit_message>
Humana payer under availity wired up
</commit_message>
<xml_diff>
--- a/backend/src/workflows/claim-status/portals/availity/config/Payer_mapping_ava.xlsx
+++ b/backend/src/workflows/claim-status/portals/availity/config/Payer_mapping_ava.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alamelu\Documents\Repos\claim-status-check\backend\src\scrapers\availity\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alamelu\Documents\Repos\claim-status-check\backend\src\workflows\claim-status\portals\availity\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31F17329-0A11-4F70-A1B4-7FDD1D18E3BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB3567A-2312-41F9-8621-A79722FF7FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{4DE94660-A54E-46F6-AD6A-893CA67AF137}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
   <si>
     <t xml:space="preserve">Payer name in excel </t>
   </si>
@@ -64,6 +64,12 @@
   </si>
   <si>
     <t>WELLCARE</t>
+  </si>
+  <si>
+    <t>Humana gold Plus</t>
+  </si>
+  <si>
+    <t>HUMANA</t>
   </si>
 </sst>
 </file>
@@ -415,7 +421,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B88755D1-98D7-4BD5-87AA-1A7D67B6D9D9}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47" customWidth="1"/>
@@ -478,6 +484,22 @@
         <v>12</v>
       </c>
     </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Started availity for medrevenu and added Anthem CA payer
</commit_message>
<xml_diff>
--- a/backend/src/workflows/claim-status/portals/availity/config/Payer_mapping_ava.xlsx
+++ b/backend/src/workflows/claim-status/portals/availity/config/Payer_mapping_ava.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alamelu\Documents\Repos\claim-status-check\backend\src\workflows\claim-status\portals\availity\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB3567A-2312-41F9-8621-A79722FF7FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95E6A7B3-AF72-488D-92EA-A07354045DF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{4DE94660-A54E-46F6-AD6A-893CA67AF137}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
   <si>
     <t xml:space="preserve">Payer name in excel </t>
   </si>
@@ -70,19 +70,31 @@
   </si>
   <si>
     <t>HUMANA</t>
+  </si>
+  <si>
+    <t>1 - BLUE CROSS OF CALIFORNIA</t>
+  </si>
+  <si>
+    <t>ANTHEM - CA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF242424"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -105,8 +117,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -421,7 +434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B88755D1-98D7-4BD5-87AA-1A7D67B6D9D9}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47" customWidth="1"/>
@@ -500,6 +513,14 @@
         <v>14</v>
       </c>
     </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Molina payer added under availity
</commit_message>
<xml_diff>
--- a/backend/src/workflows/claim-status/portals/availity/config/Payer_mapping_ava.xlsx
+++ b/backend/src/workflows/claim-status/portals/availity/config/Payer_mapping_ava.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alamelu\Documents\Repos\claim-status-check\backend\src\workflows\claim-status\portals\availity\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95E6A7B3-AF72-488D-92EA-A07354045DF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85C4620A-B206-4DF3-A29C-8DDEDE533410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{4DE94660-A54E-46F6-AD6A-893CA67AF137}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="25">
   <si>
     <t xml:space="preserve">Payer name in excel </t>
   </si>
@@ -76,13 +76,37 @@
   </si>
   <si>
     <t>ANTHEM - CA</t>
+  </si>
+  <si>
+    <t>MOLINA HEALTHCARE CALIFORNIA</t>
+  </si>
+  <si>
+    <t>2 - MOLINA (MCAL)</t>
+  </si>
+  <si>
+    <t>2 - MOLINA</t>
+  </si>
+  <si>
+    <t>1 - MOLINA (MCAL)</t>
+  </si>
+  <si>
+    <t>1 - MOLINA</t>
+  </si>
+  <si>
+    <t>2 - MOLINA MEDICAL GROUP</t>
+  </si>
+  <si>
+    <t>2 - MOLINA ADVANTAGE(MCARE)</t>
+  </si>
+  <si>
+    <t>2 - MOLINA HEALTHCARE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -95,6 +119,13 @@
       <color rgb="FF242424"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -117,9 +148,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -434,11 +469,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B88755D1-98D7-4BD5-87AA-1A7D67B6D9D9}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47" customWidth="1"/>
     <col min="2" max="2" width="34.140625" customWidth="1"/>
+    <col min="6" max="8" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -521,6 +557,65 @@
         <v>16</v>
       </c>
     </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Medrevenu 4 payers done with service date tab
</commit_message>
<xml_diff>
--- a/backend/src/workflows/claim-status/portals/availity/config/Payer_mapping_ava.xlsx
+++ b/backend/src/workflows/claim-status/portals/availity/config/Payer_mapping_ava.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alamelu\Documents\Repos\claim-status-check\backend\src\workflows\claim-status\portals\availity\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85C4620A-B206-4DF3-A29C-8DDEDE533410}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFDF1E1F-C647-4451-B6BF-ACE1369613E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{4DE94660-A54E-46F6-AD6A-893CA67AF137}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="52">
   <si>
     <t xml:space="preserve">Payer name in excel </t>
   </si>
@@ -100,13 +100,94 @@
   </si>
   <si>
     <t>2 - MOLINA HEALTHCARE</t>
+  </si>
+  <si>
+    <t>1 - HEALTH NET IFP ENHANCED CARE PPO</t>
+  </si>
+  <si>
+    <t>1 - HEALTH NET</t>
+  </si>
+  <si>
+    <t>1 - HEALTH NET COMMERCIAL</t>
+  </si>
+  <si>
+    <t>1 - HEALTH NET COMMERCIAL CLAIMS</t>
+  </si>
+  <si>
+    <t>1 - HEALTH NET HMO DIRECT NETWORK</t>
+  </si>
+  <si>
+    <t>1 - HEALTH NET PPO</t>
+  </si>
+  <si>
+    <t>1 - HEALTH NET MEDI-CAL</t>
+  </si>
+  <si>
+    <t>1 - HEALTH NET - COMM</t>
+  </si>
+  <si>
+    <t>2 - HEALTH NET</t>
+  </si>
+  <si>
+    <t>1 - HEALTH NET FEDERAL SERVICES</t>
+  </si>
+  <si>
+    <t>2 - HEALTH NET IFP ENHANCED CARE PPO</t>
+  </si>
+  <si>
+    <t>2 - HEALTH NET - COMM</t>
+  </si>
+  <si>
+    <t>2 - HEALTH NET HMO DIRECT NETWORK</t>
+  </si>
+  <si>
+    <t>1 - HEALTH NET FEDERAL SERVICES, LLC</t>
+  </si>
+  <si>
+    <t>HEALTH NET</t>
+  </si>
+  <si>
+    <t>1 - HUMANA</t>
+  </si>
+  <si>
+    <t>1 - HUMANA CHOICE CARE PPO</t>
+  </si>
+  <si>
+    <t>2 - HUMANA CHOICE CARE PPO</t>
+  </si>
+  <si>
+    <t>2 - HUMANA</t>
+  </si>
+  <si>
+    <t>TRIWEST - TRICARE</t>
+  </si>
+  <si>
+    <t>1 - TRIWEST HEALTHCARE ALLIANCE</t>
+  </si>
+  <si>
+    <t>1 - TRICARE WEST REGION CLAIMS</t>
+  </si>
+  <si>
+    <t>1 - TRICARE WEST CLAIM</t>
+  </si>
+  <si>
+    <t>1 - TRICARE WEST</t>
+  </si>
+  <si>
+    <t>3 - TRICARE WEST CLAIM</t>
+  </si>
+  <si>
+    <t>1 - TRIWEST-TRICARE WEST REGION</t>
+  </si>
+  <si>
+    <t>2 - TRIWEST HEALTHCARE ALLIANCE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -126,6 +207,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -148,13 +235,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -469,7 +559,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B88755D1-98D7-4BD5-87AA-1A7D67B6D9D9}">
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47" customWidth="1"/>
@@ -614,7 +704,204 @@
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="3"/>
+      <c r="A18" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B18" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B24" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B27" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B30" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B31" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>40</v>
+      </c>
+      <c r="B32" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>41</v>
+      </c>
+      <c r="B33" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B34" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B35" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B36" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B37" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B38" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B39" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B40" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B41" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B42" t="s">
+        <v>44</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>